<commit_message>
Add/Update Quantities.xlsx via API
</commit_message>
<xml_diff>
--- a/Quantities.xlsx
+++ b/Quantities.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L525"/>
+  <dimension ref="A1:L528"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17973,6 +17973,100 @@
       <c r="K525" t="inlineStr"/>
       <c r="L525" t="inlineStr"/>
     </row>
+    <row r="526">
+      <c r="A526" s="2" t="n">
+        <v>46082</v>
+      </c>
+      <c r="B526" t="n">
+        <v>0.00018791</v>
+      </c>
+      <c r="C526" t="n">
+        <v>7.45e-06</v>
+      </c>
+      <c r="D526" t="n">
+        <v>3.635e-05</v>
+      </c>
+      <c r="E526" t="n">
+        <v>465.80531254</v>
+      </c>
+      <c r="F526" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G526" t="n">
+        <v>0.0004431</v>
+      </c>
+      <c r="H526" t="n">
+        <v>5691.42185423</v>
+      </c>
+      <c r="I526" t="n">
+        <v>0.008201770000000001</v>
+      </c>
+      <c r="J526" t="inlineStr"/>
+      <c r="K526" t="inlineStr"/>
+      <c r="L526" t="inlineStr"/>
+    </row>
+    <row r="527">
+      <c r="A527" s="2" t="n">
+        <v>46083</v>
+      </c>
+      <c r="B527" t="n">
+        <v>0.00018791</v>
+      </c>
+      <c r="C527" t="n">
+        <v>7.45e-06</v>
+      </c>
+      <c r="D527" t="n">
+        <v>3.635e-05</v>
+      </c>
+      <c r="E527" t="n">
+        <v>465.80531254</v>
+      </c>
+      <c r="F527" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G527" t="n">
+        <v>0.0004431</v>
+      </c>
+      <c r="H527" t="n">
+        <v>5691.42185423</v>
+      </c>
+      <c r="I527" t="n">
+        <v>0.008201770000000001</v>
+      </c>
+      <c r="J527" t="inlineStr"/>
+      <c r="K527" t="inlineStr"/>
+      <c r="L527" t="inlineStr"/>
+    </row>
+    <row r="528">
+      <c r="A528" s="2" t="n">
+        <v>46084</v>
+      </c>
+      <c r="B528" t="n">
+        <v>0.00018791</v>
+      </c>
+      <c r="C528" t="n">
+        <v>7.45e-06</v>
+      </c>
+      <c r="D528" t="n">
+        <v>3.635e-05</v>
+      </c>
+      <c r="E528" t="inlineStr"/>
+      <c r="F528" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G528" t="n">
+        <v>0.0004431</v>
+      </c>
+      <c r="H528" t="n">
+        <v>5691.42185423</v>
+      </c>
+      <c r="I528" t="n">
+        <v>0.008201770000000001</v>
+      </c>
+      <c r="J528" t="inlineStr"/>
+      <c r="K528" t="inlineStr"/>
+      <c r="L528" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>